<commit_message>
The Math excel and img's, chron updates
</commit_message>
<xml_diff>
--- a/excel/Colorado_River_Notes.xlsx
+++ b/excel/Colorado_River_Notes.xlsx
@@ -11,11 +11,16 @@
     <sheet name="Notes" sheetId="1" state="visible" r:id="rId2"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <extLst>
+    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
+      <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="22">
   <si>
     <t xml:space="preserve">Color</t>
   </si>
@@ -41,19 +46,37 @@
     <t xml:space="preserve">USBR Lower Basin Annual Reports Consumptive Use</t>
   </si>
   <si>
-    <t xml:space="preserve">USBR Lower Basin Annual Flow</t>
-  </si>
-  <si>
-    <t xml:space="preserve">USBR Upper Basin Consumptive Use Loss Report</t>
+    <t xml:space="preserve">data/USBR_Reports/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USBR Lower Basin Annual Report Flow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USBR Upper Basin Consumptive Uses and Losses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data/Colorado_River/V24.5_CUL_ResultsCU_CY.xlsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AF/MAF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USBR Lower Basin Consumptive Uses and Losses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data/Colorado_River/1971-2024 Lower Colorado River System CUL Data.xlsx</t>
   </si>
   <si>
     <t xml:space="preserve">USBR Natural Flow</t>
   </si>
   <si>
-    <t xml:space="preserve">WY</t>
+    <t xml:space="preserve">data/Colorado_River/NaturalFlows1906-2020_20221215.xlsx</t>
   </si>
   <si>
     <t xml:space="preserve">USGS Gage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API</t>
   </si>
   <si>
     <t xml:space="preserve">USBR RISE</t>
@@ -72,11 +95,12 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -93,8 +117,13 @@
       <name val="Arial"/>
       <family val="0"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -115,8 +144,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFD28C"/>
+        <bgColor rgb="FFFFB66C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFB66C"/>
-        <bgColor rgb="FFFF99CC"/>
+        <bgColor rgb="FFFFD28C"/>
       </patternFill>
     </fill>
     <fill>
@@ -269,7 +304,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -322,6 +357,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -339,6 +378,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="8" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -418,9 +461,9 @@
       <rgbColor rgb="FFCCFFCC"/>
       <rgbColor rgb="FFFFE6E6"/>
       <rgbColor rgb="FF99CCFF"/>
-      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFFFB66C"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFB66C"/>
+      <rgbColor rgb="FFFFD28C"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
@@ -447,8 +490,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:O51"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="B1:O52"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="5.4"/>
   </cols>
@@ -506,6 +549,9 @@
       <c r="E3" s="0" t="s">
         <v>7</v>
       </c>
+      <c r="I3" s="0" t="s">
+        <v>8</v>
+      </c>
       <c r="O3" s="10"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -517,14 +563,17 @@
         <v>6</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F4" s="12"/>
       <c r="G4" s="12"/>
+      <c r="I4" s="13" t="s">
+        <v>8</v>
+      </c>
       <c r="O4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="13"/>
+      <c r="B5" s="14"/>
       <c r="C5" s="9" t="s">
         <v>5</v>
       </c>
@@ -532,271 +581,304 @@
         <v>6</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F5" s="12"/>
       <c r="G5" s="12"/>
+      <c r="I5" s="13" t="s">
+        <v>11</v>
+      </c>
       <c r="O5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="14"/>
+      <c r="B6" s="15"/>
       <c r="C6" s="9" t="s">
         <v>5</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F6" s="12"/>
       <c r="G6" s="12"/>
+      <c r="I6" s="13" t="s">
+        <v>14</v>
+      </c>
       <c r="O6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="15"/>
+      <c r="B7" s="16"/>
       <c r="C7" s="9" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="D7" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="E7" s="0" t="s">
-        <v>12</v>
+      <c r="E7" s="12" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="12"/>
+      <c r="G7" s="12"/>
+      <c r="I7" s="13" t="s">
+        <v>16</v>
       </c>
       <c r="O7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="16"/>
+      <c r="B8" s="17"/>
       <c r="C8" s="9" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="D8" s="9" t="s">
         <v>6</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>13</v>
+        <v>17</v>
+      </c>
+      <c r="I8" s="0" t="s">
+        <v>18</v>
       </c>
       <c r="O8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="17"/>
+      <c r="B9" s="18"/>
       <c r="C9" s="9" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>15</v>
+        <v>19</v>
+      </c>
+      <c r="I9" s="0" t="s">
+        <v>18</v>
       </c>
       <c r="O9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="18"/>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
+      <c r="B10" s="19"/>
+      <c r="C10" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="E10" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="I10" s="0" t="s">
+        <v>18</v>
+      </c>
       <c r="O10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="18"/>
+      <c r="B11" s="20"/>
       <c r="C11" s="9"/>
       <c r="D11" s="9"/>
       <c r="O11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="18"/>
+      <c r="B12" s="20"/>
       <c r="C12" s="9"/>
       <c r="D12" s="9"/>
       <c r="O12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="19"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="21"/>
-      <c r="F13" s="21"/>
-      <c r="G13" s="21"/>
-      <c r="H13" s="21"/>
-      <c r="I13" s="21"/>
-      <c r="J13" s="21"/>
-      <c r="K13" s="21"/>
-      <c r="L13" s="21"/>
-      <c r="M13" s="21"/>
-      <c r="N13" s="21"/>
-      <c r="O13" s="22"/>
+      <c r="B13" s="20"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="O13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="23"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
+      <c r="B14" s="21"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="23"/>
+      <c r="H14" s="23"/>
+      <c r="I14" s="23"/>
+      <c r="J14" s="23"/>
+      <c r="K14" s="23"/>
+      <c r="L14" s="23"/>
+      <c r="M14" s="23"/>
+      <c r="N14" s="23"/>
+      <c r="O14" s="24"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="23"/>
+      <c r="B15" s="25"/>
       <c r="C15" s="9"/>
       <c r="D15" s="9"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="23"/>
+      <c r="B16" s="25"/>
       <c r="C16" s="9"/>
       <c r="D16" s="9"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="23"/>
+      <c r="B17" s="25"/>
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="23"/>
+      <c r="B18" s="25"/>
       <c r="C18" s="9"/>
       <c r="D18" s="9"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="23"/>
+      <c r="B19" s="25"/>
       <c r="C19" s="9"/>
       <c r="D19" s="9"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="23"/>
+      <c r="B20" s="25"/>
       <c r="C20" s="9"/>
       <c r="D20" s="9"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="23"/>
+      <c r="B21" s="25"/>
       <c r="C21" s="9"/>
       <c r="D21" s="9"/>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="23"/>
+      <c r="B22" s="25"/>
       <c r="C22" s="9"/>
       <c r="D22" s="9"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="23"/>
+      <c r="B23" s="25"/>
       <c r="C23" s="9"/>
       <c r="D23" s="9"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="23"/>
+      <c r="B24" s="25"/>
       <c r="C24" s="9"/>
       <c r="D24" s="9"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="23"/>
+      <c r="B25" s="25"/>
       <c r="C25" s="9"/>
       <c r="D25" s="9"/>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="23"/>
+      <c r="B26" s="25"/>
       <c r="C26" s="9"/>
       <c r="D26" s="9"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="23"/>
+      <c r="B27" s="25"/>
       <c r="C27" s="9"/>
       <c r="D27" s="9"/>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="23"/>
+      <c r="B28" s="25"/>
       <c r="C28" s="9"/>
       <c r="D28" s="9"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="23"/>
+      <c r="B29" s="25"/>
       <c r="C29" s="9"/>
       <c r="D29" s="9"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="23"/>
+      <c r="B30" s="25"/>
       <c r="C30" s="9"/>
       <c r="D30" s="9"/>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="23"/>
+      <c r="B31" s="25"/>
       <c r="C31" s="9"/>
       <c r="D31" s="9"/>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="23"/>
+      <c r="B32" s="25"/>
       <c r="C32" s="9"/>
       <c r="D32" s="9"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="23"/>
+      <c r="B33" s="25"/>
       <c r="C33" s="9"/>
       <c r="D33" s="9"/>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="23"/>
+      <c r="B34" s="25"/>
       <c r="C34" s="9"/>
       <c r="D34" s="9"/>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="23"/>
+      <c r="B35" s="25"/>
       <c r="C35" s="9"/>
       <c r="D35" s="9"/>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="23"/>
+      <c r="B36" s="25"/>
       <c r="C36" s="9"/>
       <c r="D36" s="9"/>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="23"/>
+      <c r="B37" s="25"/>
       <c r="C37" s="9"/>
       <c r="D37" s="9"/>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B38" s="23"/>
+      <c r="B38" s="25"/>
       <c r="C38" s="9"/>
       <c r="D38" s="9"/>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="23"/>
+      <c r="B39" s="25"/>
       <c r="C39" s="9"/>
       <c r="D39" s="9"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="23"/>
+      <c r="B40" s="25"/>
       <c r="C40" s="9"/>
       <c r="D40" s="9"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B41" s="23"/>
+      <c r="B41" s="25"/>
       <c r="C41" s="9"/>
       <c r="D41" s="9"/>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B42" s="23"/>
+      <c r="B42" s="25"/>
       <c r="C42" s="9"/>
       <c r="D42" s="9"/>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="23"/>
+      <c r="B43" s="25"/>
+      <c r="C43" s="9"/>
+      <c r="D43" s="9"/>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="23"/>
+      <c r="B44" s="25"/>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="23"/>
+      <c r="B45" s="25"/>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B46" s="23"/>
+      <c r="B46" s="25"/>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B47" s="23"/>
+      <c r="B47" s="25"/>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B48" s="23"/>
+      <c r="B48" s="25"/>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B49" s="23"/>
+      <c r="B49" s="25"/>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B50" s="23"/>
+      <c r="B50" s="25"/>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B51" s="24"/>
+      <c r="B51" s="25"/>
+    </row>
+    <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B52" s="26"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Notes update for big river issues edition
</commit_message>
<xml_diff>
--- a/excel/Colorado_River_Notes.xlsx
+++ b/excel/Colorado_River_Notes.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="24">
   <si>
     <t xml:space="preserve">Color</t>
   </si>
@@ -61,10 +61,16 @@
     <t xml:space="preserve">AF/MAF</t>
   </si>
   <si>
-    <t xml:space="preserve">USBR Lower Basin Consumptive Uses and Losses</t>
+    <t xml:space="preserve">USBR Lower Basin Mainstream CUL</t>
   </si>
   <si>
     <t xml:space="preserve">data/Colorado_River/1971-2024 Lower Colorado River System CUL Data.xlsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USBR Lower Basin Reservoir CUL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USBR Lower Basin Tributary CUL</t>
   </si>
   <si>
     <t xml:space="preserve">USBR Natural Flow</t>
@@ -95,7 +101,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="4">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -117,13 +123,8 @@
       <name val="Arial"/>
       <family val="0"/>
     </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
   </fonts>
-  <fills count="10">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -156,6 +157,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFF6D6D"/>
+        <bgColor rgb="FFFF6600"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF6D"/>
+        <bgColor rgb="FFFFFFD0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFE8FFE0"/>
         <bgColor rgb="FFFFFFD0"/>
       </patternFill>
@@ -169,7 +182,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFE0F0FF"/>
-        <bgColor rgb="FFCCFFFF"/>
+        <bgColor rgb="FFE8FFE0"/>
       </patternFill>
     </fill>
     <fill>
@@ -304,7 +317,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -357,10 +370,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -382,6 +391,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="9" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="10" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="9" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -445,7 +462,7 @@
       <rgbColor rgb="FFFFFFD0"/>
       <rgbColor rgb="FFE0F0FF"/>
       <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FFFF6D6D"/>
       <rgbColor rgb="FF0066CC"/>
       <rgbColor rgb="FFFFE0FF"/>
       <rgbColor rgb="FF000080"/>
@@ -457,9 +474,9 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFFFE6E6"/>
       <rgbColor rgb="FFCCFFCC"/>
-      <rgbColor rgb="FFFFE6E6"/>
+      <rgbColor rgb="FFFFFF6D"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFFB66C"/>
       <rgbColor rgb="FFCC99FF"/>
@@ -490,8 +507,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B1:O52"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="B1:O54"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="5.4"/>
   </cols>
@@ -567,13 +584,13 @@
       </c>
       <c r="F4" s="12"/>
       <c r="G4" s="12"/>
-      <c r="I4" s="13" t="s">
+      <c r="I4" s="12" t="s">
         <v>8</v>
       </c>
       <c r="O4" s="10"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B5" s="14"/>
+      <c r="B5" s="13"/>
       <c r="C5" s="9" t="s">
         <v>5</v>
       </c>
@@ -585,13 +602,13 @@
       </c>
       <c r="F5" s="12"/>
       <c r="G5" s="12"/>
-      <c r="I5" s="13" t="s">
+      <c r="I5" s="12" t="s">
         <v>11</v>
       </c>
       <c r="O5" s="10"/>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B6" s="15"/>
+      <c r="B6" s="14"/>
       <c r="C6" s="9" t="s">
         <v>5</v>
       </c>
@@ -603,282 +620,318 @@
       </c>
       <c r="F6" s="12"/>
       <c r="G6" s="12"/>
-      <c r="I6" s="13" t="s">
+      <c r="I6" s="12" t="s">
         <v>14</v>
       </c>
       <c r="O6" s="10"/>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B7" s="16"/>
+      <c r="B7" s="15"/>
       <c r="C7" s="9" t="s">
         <v>5</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E7" s="12" t="s">
         <v>15</v>
       </c>
       <c r="F7" s="12"/>
       <c r="G7" s="12"/>
-      <c r="I7" s="13" t="s">
-        <v>16</v>
+      <c r="I7" s="12" t="s">
+        <v>14</v>
       </c>
       <c r="O7" s="10"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B8" s="17"/>
+      <c r="B8" s="16"/>
       <c r="C8" s="9" t="s">
         <v>5</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="E8" s="0" t="s">
-        <v>17</v>
-      </c>
-      <c r="I8" s="0" t="s">
-        <v>18</v>
+        <v>12</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" s="12"/>
+      <c r="G8" s="12"/>
+      <c r="I8" s="12" t="s">
+        <v>14</v>
       </c>
       <c r="O8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="18"/>
+      <c r="B9" s="17"/>
       <c r="C9" s="9" t="s">
         <v>5</v>
       </c>
       <c r="D9" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="E9" s="0" t="s">
-        <v>19</v>
-      </c>
-      <c r="I9" s="0" t="s">
+      <c r="E9" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
+      <c r="I9" s="12" t="s">
         <v>18</v>
       </c>
       <c r="O9" s="10"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B10" s="19"/>
+      <c r="B10" s="18"/>
       <c r="C10" s="9" t="s">
         <v>5</v>
       </c>
       <c r="D10" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="E10" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="I10" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="E10" s="0" t="s">
+      <c r="O10" s="10"/>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="19"/>
+      <c r="C11" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="E11" s="0" t="s">
         <v>21</v>
       </c>
-      <c r="I10" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="O10" s="10"/>
-    </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B11" s="20"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
+      <c r="I11" s="0" t="s">
+        <v>20</v>
+      </c>
       <c r="O11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="20"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
+      <c r="C12" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="E12" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="I12" s="0" t="s">
+        <v>20</v>
+      </c>
       <c r="O12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B13" s="20"/>
+      <c r="B13" s="21"/>
       <c r="C13" s="9"/>
       <c r="D13" s="9"/>
       <c r="O13" s="10"/>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="21"/>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
-      <c r="E14" s="23"/>
-      <c r="F14" s="23"/>
-      <c r="G14" s="23"/>
-      <c r="H14" s="23"/>
-      <c r="I14" s="23"/>
-      <c r="J14" s="23"/>
-      <c r="K14" s="23"/>
-      <c r="L14" s="23"/>
-      <c r="M14" s="23"/>
-      <c r="N14" s="23"/>
-      <c r="O14" s="24"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="O14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="25"/>
+      <c r="B15" s="21"/>
       <c r="C15" s="9"/>
       <c r="D15" s="9"/>
+      <c r="O15" s="10"/>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="25"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
+      <c r="B16" s="22"/>
+      <c r="C16" s="23"/>
+      <c r="D16" s="23"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="24"/>
+      <c r="I16" s="24"/>
+      <c r="J16" s="24"/>
+      <c r="K16" s="24"/>
+      <c r="L16" s="24"/>
+      <c r="M16" s="24"/>
+      <c r="N16" s="24"/>
+      <c r="O16" s="25"/>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="25"/>
+      <c r="B17" s="26"/>
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="25"/>
+      <c r="B18" s="26"/>
       <c r="C18" s="9"/>
       <c r="D18" s="9"/>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="25"/>
+      <c r="B19" s="26"/>
       <c r="C19" s="9"/>
       <c r="D19" s="9"/>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="25"/>
+      <c r="B20" s="26"/>
       <c r="C20" s="9"/>
       <c r="D20" s="9"/>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B21" s="25"/>
+      <c r="B21" s="26"/>
       <c r="C21" s="9"/>
       <c r="D21" s="9"/>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="25"/>
+      <c r="B22" s="26"/>
       <c r="C22" s="9"/>
       <c r="D22" s="9"/>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="25"/>
+      <c r="B23" s="26"/>
       <c r="C23" s="9"/>
       <c r="D23" s="9"/>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="25"/>
+      <c r="B24" s="26"/>
       <c r="C24" s="9"/>
       <c r="D24" s="9"/>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="25"/>
+      <c r="B25" s="26"/>
       <c r="C25" s="9"/>
       <c r="D25" s="9"/>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="25"/>
+      <c r="B26" s="26"/>
       <c r="C26" s="9"/>
       <c r="D26" s="9"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="25"/>
+      <c r="B27" s="26"/>
       <c r="C27" s="9"/>
       <c r="D27" s="9"/>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="25"/>
+      <c r="B28" s="26"/>
       <c r="C28" s="9"/>
       <c r="D28" s="9"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="25"/>
+      <c r="B29" s="26"/>
       <c r="C29" s="9"/>
       <c r="D29" s="9"/>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="25"/>
+      <c r="B30" s="26"/>
       <c r="C30" s="9"/>
       <c r="D30" s="9"/>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="25"/>
+      <c r="B31" s="26"/>
       <c r="C31" s="9"/>
       <c r="D31" s="9"/>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="25"/>
+      <c r="B32" s="26"/>
       <c r="C32" s="9"/>
       <c r="D32" s="9"/>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="25"/>
+      <c r="B33" s="26"/>
       <c r="C33" s="9"/>
       <c r="D33" s="9"/>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B34" s="25"/>
+      <c r="B34" s="26"/>
       <c r="C34" s="9"/>
       <c r="D34" s="9"/>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="25"/>
+      <c r="B35" s="26"/>
       <c r="C35" s="9"/>
       <c r="D35" s="9"/>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="25"/>
+      <c r="B36" s="26"/>
       <c r="C36" s="9"/>
       <c r="D36" s="9"/>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="25"/>
+      <c r="B37" s="26"/>
       <c r="C37" s="9"/>
       <c r="D37" s="9"/>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B38" s="25"/>
+      <c r="B38" s="26"/>
       <c r="C38" s="9"/>
       <c r="D38" s="9"/>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="25"/>
+      <c r="B39" s="26"/>
       <c r="C39" s="9"/>
       <c r="D39" s="9"/>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="25"/>
+      <c r="B40" s="26"/>
       <c r="C40" s="9"/>
       <c r="D40" s="9"/>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B41" s="25"/>
+      <c r="B41" s="26"/>
       <c r="C41" s="9"/>
       <c r="D41" s="9"/>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B42" s="25"/>
+      <c r="B42" s="26"/>
       <c r="C42" s="9"/>
       <c r="D42" s="9"/>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="25"/>
+      <c r="B43" s="26"/>
       <c r="C43" s="9"/>
       <c r="D43" s="9"/>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="25"/>
+      <c r="B44" s="26"/>
+      <c r="C44" s="9"/>
+      <c r="D44" s="9"/>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="25"/>
+      <c r="B45" s="26"/>
+      <c r="C45" s="9"/>
+      <c r="D45" s="9"/>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B46" s="25"/>
+      <c r="B46" s="26"/>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B47" s="25"/>
+      <c r="B47" s="26"/>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B48" s="25"/>
+      <c r="B48" s="26"/>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B49" s="25"/>
+      <c r="B49" s="26"/>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B50" s="25"/>
+      <c r="B50" s="26"/>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B51" s="25"/>
+      <c r="B51" s="26"/>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="26"/>
+    </row>
+    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B53" s="26"/>
+    </row>
+    <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B54" s="27"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>